<commit_message>
docs(bom): remove M8 Washer (no longer used)
Drop M8 Washer from the fastener matrix on the page and from the
spreadsheet's Nuts&Bolts-List -- it was unused (zero across every assembly).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/assets/BoM.xlsx
+++ b/docs/assets/BoM.xlsx
@@ -132,7 +132,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -286,12 +286,56 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -374,6 +418,8 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -803,8 +849,8 @@
           <t>Circuit</t>
         </is>
       </c>
-      <c r="B2" s="45" t="n"/>
-      <c r="C2" s="45" t="n"/>
+      <c r="B2" s="64" t="n"/>
+      <c r="C2" s="65" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="46" t="inlineStr">
@@ -1011,8 +1057,8 @@
           <t>Mount</t>
         </is>
       </c>
-      <c r="B16" s="45" t="n"/>
-      <c r="C16" s="45" t="n"/>
+      <c r="B16" s="64" t="n"/>
+      <c r="C16" s="65" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="46" t="inlineStr">
@@ -1230,8 +1276,8 @@
           <t>Mount - HDMI</t>
         </is>
       </c>
-      <c r="B31" s="45" t="n"/>
-      <c r="C31" s="45" t="n"/>
+      <c r="B31" s="64" t="n"/>
+      <c r="C31" s="65" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="46" t="inlineStr">
@@ -1269,8 +1315,8 @@
           <t>Mount - SDI</t>
         </is>
       </c>
-      <c r="B34" s="45" t="n"/>
-      <c r="C34" s="45" t="n"/>
+      <c r="B34" s="64" t="n"/>
+      <c r="C34" s="65" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="46" t="inlineStr">
@@ -1308,8 +1354,8 @@
           <t>Mount - BMD Converter</t>
         </is>
       </c>
-      <c r="B37" s="45" t="n"/>
-      <c r="C37" s="45" t="n"/>
+      <c r="B37" s="64" t="n"/>
+      <c r="C37" s="65" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="46" t="inlineStr">
@@ -1377,8 +1423,8 @@
           <t>Slider</t>
         </is>
       </c>
-      <c r="B42" s="45" t="n"/>
-      <c r="C42" s="45" t="n"/>
+      <c r="B42" s="64" t="n"/>
+      <c r="C42" s="65" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="46" t="inlineStr">
@@ -1523,8 +1569,8 @@
           <t>Slider - HDMI</t>
         </is>
       </c>
-      <c r="B52" s="45" t="n"/>
-      <c r="C52" s="45" t="n"/>
+      <c r="B52" s="64" t="n"/>
+      <c r="C52" s="65" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="46" t="inlineStr">
@@ -1562,8 +1608,8 @@
           <t>Slider - SDI</t>
         </is>
       </c>
-      <c r="B55" s="45" t="n"/>
-      <c r="C55" s="45" t="n"/>
+      <c r="B55" s="64" t="n"/>
+      <c r="C55" s="65" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="46" t="inlineStr">
@@ -1601,8 +1647,8 @@
           <t>Slider - BMD Converter</t>
         </is>
       </c>
-      <c r="B58" s="45" t="n"/>
-      <c r="C58" s="45" t="n"/>
+      <c r="B58" s="64" t="n"/>
+      <c r="C58" s="65" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="46" t="inlineStr">
@@ -1640,8 +1686,8 @@
           <t>Hub</t>
         </is>
       </c>
-      <c r="B61" s="45" t="n"/>
-      <c r="C61" s="45" t="n"/>
+      <c r="B61" s="64" t="n"/>
+      <c r="C61" s="65" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="46" t="inlineStr">
@@ -1664,8 +1710,8 @@
           <t>Hub Display</t>
         </is>
       </c>
-      <c r="B63" s="45" t="n"/>
-      <c r="C63" s="45" t="n"/>
+      <c r="B63" s="64" t="n"/>
+      <c r="C63" s="65" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="46" t="inlineStr">
@@ -1733,8 +1779,8 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="B68" s="45" t="n"/>
-      <c r="C68" s="45" t="n"/>
+      <c r="B68" s="64" t="n"/>
+      <c r="C68" s="65" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="46" t="inlineStr">
@@ -1772,8 +1818,8 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="B71" s="45" t="n"/>
-      <c r="C71" s="45" t="n"/>
+      <c r="B71" s="64" t="n"/>
+      <c r="C71" s="65" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="46" t="inlineStr">
@@ -1876,7 +1922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS57"/>
+  <dimension ref="A1:AN57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="10.83203125" customWidth="1" style="19" min="1" max="1"/>
@@ -2966,7 +3012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="3.33203125" customWidth="1" min="1" max="1"/>
@@ -4092,35 +4138,6 @@
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="62" t="inlineStr">
-        <is>
-          <t>M8 Washer</t>
-        </is>
-      </c>
-      <c r="C34" s="47" t="n"/>
-      <c r="D34" s="47" t="n"/>
-      <c r="E34" s="47" t="n"/>
-      <c r="F34" s="47" t="n"/>
-      <c r="G34" s="47" t="n"/>
-      <c r="H34" s="47" t="n"/>
-      <c r="I34" s="47" t="n"/>
-      <c r="J34" s="47" t="n"/>
-      <c r="K34" s="47" t="n"/>
-      <c r="L34" s="47" t="n"/>
-      <c r="M34" s="47" t="n"/>
-      <c r="N34" s="47" t="n"/>
-      <c r="O34" s="47" t="n"/>
-      <c r="P34" s="47" t="n"/>
-      <c r="Q34" s="47" t="n"/>
-      <c r="R34" s="47" t="n"/>
-      <c r="S34" s="47" t="n"/>
-      <c r="T34" s="47" t="n"/>
-      <c r="U34" s="63">
-        <f>SUM(C34:T34)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: correct the UNC tripod fasteners to 1/4"
They were recorded inconsistently as 3/8 UNC inserts and a "3/4 UNC 40mm"
bolt, with the matrix calling the same bolt "UNC x 40". They are all 1/4 UNC
tripod threads, and the bolt is 1½ inches, not 40 mm. Seven cells across both
sheets now read "1/4 UNC Insert" and "1/4 UNC x 1½"", so the two sheets agree
and the page regenerates from them.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/assets/BoM.xlsx
+++ b/docs/assets/BoM.xlsx
@@ -1907,7 +1907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AN57"/>
+  <dimension ref="A1:AN57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="10.83203125" customWidth="1" style="41" min="1" max="1"/>
@@ -1949,6 +1949,7 @@
     <col width="10.83203125" customWidth="1" style="41" min="40" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="18" t="inlineStr">
         <is>
@@ -2157,7 +2158,7 @@
       </c>
       <c r="AD4" s="38" t="inlineStr">
         <is>
-          <t>3/8 UNC Insert</t>
+          <t>1/4 UNC Insert</t>
         </is>
       </c>
       <c r="AE4" s="40" t="n">
@@ -2469,6 +2470,10 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="B20" s="18" t="inlineStr">
         <is>
@@ -2528,7 +2533,7 @@
       <c r="D21" s="2" t="n"/>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>3/8 UNC Insert</t>
+          <t>1/4 UNC Insert</t>
         </is>
       </c>
       <c r="G21" s="20" t="n">
@@ -2591,7 +2596,7 @@
       <c r="AF21" s="2" t="n"/>
       <c r="AH21" s="39" t="inlineStr">
         <is>
-          <t>3/8 UNC Insert</t>
+          <t>1/4 UNC Insert</t>
         </is>
       </c>
       <c r="AI21" s="20" t="n">
@@ -2629,7 +2634,7 @@
     <row r="23">
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>3/8 UNC Insert</t>
+          <t>1/4 UNC Insert</t>
         </is>
       </c>
       <c r="C23" s="40" t="n">
@@ -2709,7 +2714,7 @@
       <c r="AF23" s="10" t="n"/>
       <c r="AH23" s="43" t="inlineStr">
         <is>
-          <t>3/4 UNC 40mm</t>
+          <t>1/4 UNC x 1½"</t>
         </is>
       </c>
       <c r="AI23" s="28" t="n">
@@ -3036,7 +3041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V35"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="3.33203125" customWidth="1" min="1" max="1"/>
@@ -3045,6 +3050,7 @@
     <col width="8" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="57" customHeight="1">
       <c r="B2" s="30" t="inlineStr">
         <is>
@@ -3778,7 +3784,7 @@
     <row r="22">
       <c r="B22" s="45" t="inlineStr">
         <is>
-          <t>UNC x 40</t>
+          <t>1/4 UNC x 1½"</t>
         </is>
       </c>
       <c r="C22" s="16" t="n"/>
@@ -4104,7 +4110,7 @@
     <row r="32">
       <c r="B32" s="31" t="inlineStr">
         <is>
-          <t>3/8 UNC Insert</t>
+          <t>1/4 UNC Insert</t>
         </is>
       </c>
       <c r="C32" s="16" t="n"/>

</xml_diff>

<commit_message>
docs: list the 1/4 UNC tripod fasteners in the parts list
They appeared in the fastener matrix but had no line item, so there was
nothing to order against. Quantities split by where the matrix uses them:
Mount 1 insert; Slider 4 inserts (rail ends + slider tripod mount) and 2 of
the 1½" bolts. The sheet already repeats shared items across sections, as the
GX12 connectors do. The bolt has no supplier link yet and shows a dash.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/assets/BoM.xlsx
+++ b/docs/assets/BoM.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -117,8 +117,31 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -146,8 +169,18 @@
         <fgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -331,11 +364,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -405,6 +452,28 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -803,8 +872,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <dimension ref="A1:C75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -812,1010 +881,1055 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="47" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="47" t="inlineStr">
         <is>
           <t>Buy</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="48" t="inlineStr">
         <is>
           <t>Circuit</t>
         </is>
       </c>
-      <c r="B2" s="34" t="n"/>
-      <c r="C2" s="35" t="n"/>
+      <c r="B2" s="49" t="n"/>
+      <c r="C2" s="49" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="50" t="inlineStr">
         <is>
           <t>Teensy 4.1</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="B3" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>TMC2209</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="B4" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="50" t="inlineStr">
         <is>
           <t>5V regulator</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="B5" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="50" t="inlineStr">
         <is>
           <t>1n4007</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="B6" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
         <is>
           <t>100nf 35v</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="51" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="50" t="inlineStr">
         <is>
           <t>1K ¼W</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="B8" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="50" t="inlineStr">
         <is>
           <t>100K ¼W</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="B9" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="50" t="inlineStr">
         <is>
           <t>Screw PCB terminals 5.08mm 2pin</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="B10" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="50" t="inlineStr">
         <is>
           <t>JST 4pin Plug + Lead + Socket</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="51" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>JST 5pin Plug + Lead + Socket</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="B12" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="50" t="inlineStr">
         <is>
           <t>JST 2pin Plug + Lead + Socket</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="B13" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="50" t="inlineStr">
         <is>
           <t>Header Sockets</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="51" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="50" t="inlineStr">
         <is>
           <t>Header Pins</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="51" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="A16" s="48" t="inlineStr">
         <is>
           <t>Mount</t>
         </is>
       </c>
-      <c r="B16" s="34" t="n"/>
-      <c r="C16" s="35" t="n"/>
+      <c r="B16" s="49" t="n"/>
+      <c r="C16" s="49" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="50" t="inlineStr">
         <is>
           <t>6824ZZ 120x150x16mm Bearing</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="B17" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="52" t="inlineStr">
         <is>
           <t>Simply Bearings</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="50" t="inlineStr">
         <is>
           <t>F688ZZ Flanged Bearing 8 x 16 x 5mm</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="B18" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="50" t="inlineStr">
         <is>
           <t>GT2 Pulley - 120 tooth, 8mm bore</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="B19" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="50" t="inlineStr">
         <is>
           <t>GT2 Pulley - 36 tooth, 5mm bore</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="B20" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="50" t="inlineStr">
         <is>
           <t>GT2 Pulley - 16 tooth, 5mm bore</t>
         </is>
       </c>
-      <c r="B21" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="B21" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="50" t="inlineStr">
         <is>
           <t>GT2 Belt - 580mm loop, 6mm wide</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="B22" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="50" t="inlineStr">
         <is>
           <t>GT2 Belt - 350mm loop, 6mm wide</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="B23" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="50" t="inlineStr">
         <is>
           <t>Nema14 0.9 deg 36Ncm</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="B24" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="50" t="inlineStr">
         <is>
           <t>Nema14 Round Pancake Stepper Motor 0.9 deg</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="B25" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="50" t="inlineStr">
         <is>
           <t>GX12 2 Pin Aviation Connector &amp; Panel Socket</t>
         </is>
       </c>
-      <c r="B26" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="B26" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="50" t="inlineStr">
         <is>
           <t>Waveshare ESP32-S3 1.75inch AMOLED Round Touch Display</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="B27" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="50" t="inlineStr">
         <is>
           <t>Sticky Pads Heavy Duty 40x40mm</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
+      <c r="B28" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="50" t="inlineStr">
         <is>
           <t>2.4GHz Antenna</t>
         </is>
       </c>
-      <c r="B29" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="B29" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="50" t="inlineStr">
         <is>
           <t>U.FL Mini PCI to SMA Female 20cm Lead</t>
         </is>
       </c>
-      <c r="B30" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="B30" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="33" t="inlineStr">
+      <c r="A31" s="50" t="inlineStr">
+        <is>
+          <t>1/4 UNC Insert</t>
+        </is>
+      </c>
+      <c r="B31" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="48" t="inlineStr">
         <is>
           <t>Mount - HDMI</t>
         </is>
       </c>
-      <c r="B31" s="34" t="n"/>
-      <c r="C31" s="35" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="B32" s="49" t="n"/>
+      <c r="C32" s="49" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="50" t="inlineStr">
         <is>
           <t>HDMI Keystone coupler</t>
         </is>
       </c>
-      <c r="B32" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="B33" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
         <is>
           <t>HDMI Cable - 1m</t>
         </is>
       </c>
-      <c r="B33" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="33" t="inlineStr">
+      <c r="B34" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
         <is>
           <t>Mount - SDI</t>
         </is>
       </c>
-      <c r="B34" s="34" t="n"/>
-      <c r="C34" s="35" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="B35" s="49" t="n"/>
+      <c r="C35" s="49" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="50" t="inlineStr">
         <is>
           <t>SDI Panel mount coupler</t>
         </is>
       </c>
-      <c r="B35" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="B36" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
         <is>
           <t>HD-SDI Cable - 1m</t>
         </is>
       </c>
-      <c r="B36" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="33" t="inlineStr">
+      <c r="B37" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="inlineStr">
         <is>
           <t>Mount - BMD Converter</t>
         </is>
       </c>
-      <c r="B37" s="34" t="n"/>
-      <c r="C37" s="35" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="B38" s="49" t="n"/>
+      <c r="C38" s="49" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="50" t="inlineStr">
         <is>
           <t>Blackmagic Design Bi-Directional SDI/HDMI 3G</t>
         </is>
       </c>
-      <c r="B38" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="B39" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="52" t="inlineStr">
         <is>
           <t>Thomann</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="50" t="inlineStr">
         <is>
           <t>SDI Panel mount coupler</t>
         </is>
       </c>
-      <c r="B39" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="B40" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="50" t="inlineStr">
         <is>
           <t>HD-SDI Cable - 1m, Right angle</t>
         </is>
       </c>
-      <c r="B40" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C40" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+      <c r="B41" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="50" t="inlineStr">
         <is>
           <t>USB-C Cable - 1 Metre (cut and soldered to JST 2pin)</t>
         </is>
       </c>
-      <c r="B41" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="33" t="inlineStr">
+      <c r="B42" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="48" t="inlineStr">
         <is>
           <t>Slider</t>
         </is>
       </c>
-      <c r="B42" s="34" t="n"/>
-      <c r="C42" s="35" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="B43" s="49" t="n"/>
+      <c r="C43" s="49" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="50" t="inlineStr">
         <is>
           <t>Aluminium Extrusion - 8040 C</t>
         </is>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B44" s="51" t="inlineStr">
         <is>
           <t>1000 - 3000mm</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C44" s="52" t="inlineStr">
         <is>
           <t>Ooznest</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="50" t="inlineStr">
         <is>
           <t>GT2 Pulley - 36 tooth</t>
         </is>
       </c>
-      <c r="B44" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="B45" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="50" t="inlineStr">
         <is>
           <t>GT2 Belt - 5m</t>
         </is>
       </c>
-      <c r="B45" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="B46" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="50" t="inlineStr">
         <is>
           <t>Idler - 6mm width, 3mm bore, 13mm diameter</t>
         </is>
       </c>
-      <c r="B46" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="B47" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="50" t="inlineStr">
         <is>
           <t>Nema14 1.8 deg 65Ncm</t>
         </is>
       </c>
-      <c r="B47" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="15" t="inlineStr">
+      <c r="B48" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="50" t="inlineStr">
         <is>
           <t>V Slot Pulley Wheels 625zz</t>
         </is>
       </c>
-      <c r="B48" s="16" t="n">
+      <c r="B49" s="51" t="n">
         <v>16</v>
       </c>
-      <c r="C48" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="15" t="inlineStr">
+      <c r="C49" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="50" t="inlineStr">
         <is>
           <t>XT60 Plug Connector Female and Male</t>
         </is>
       </c>
-      <c r="B49" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr">
+      <c r="B50" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="50" t="inlineStr">
         <is>
           <t>GX12 2 Pin Aviation Connector &amp; Panel Socket</t>
         </is>
       </c>
-      <c r="B50" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+      <c r="B51" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="50" t="inlineStr">
         <is>
           <t>GX12 4 Pin Aviation Connector &amp; Panel Socket</t>
         </is>
       </c>
-      <c r="B51" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="33" t="inlineStr">
+      <c r="B52" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="50" t="inlineStr">
+        <is>
+          <t>1/4 UNC Insert</t>
+        </is>
+      </c>
+      <c r="B53" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C53" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="50" t="inlineStr">
+        <is>
+          <t>1/4 UNC x 1½"</t>
+        </is>
+      </c>
+      <c r="B54" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" s="53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="48" t="inlineStr">
         <is>
           <t>Slider - HDMI</t>
         </is>
       </c>
-      <c r="B52" s="34" t="n"/>
-      <c r="C52" s="35" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="B55" s="49" t="n"/>
+      <c r="C55" s="49" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="50" t="inlineStr">
         <is>
           <t>HDMI Keystone coupler</t>
         </is>
       </c>
-      <c r="B53" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C53" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="15" t="inlineStr">
+      <c r="B56" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="50" t="inlineStr">
         <is>
           <t>HDMI Cable, 2m - 4m</t>
         </is>
       </c>
-      <c r="B54" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="33" t="inlineStr">
+      <c r="B57" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="48" t="inlineStr">
         <is>
           <t>Slider - SDI</t>
         </is>
       </c>
-      <c r="B55" s="34" t="n"/>
-      <c r="C55" s="35" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="15" t="inlineStr">
+      <c r="B58" s="49" t="n"/>
+      <c r="C58" s="49" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="50" t="inlineStr">
         <is>
           <t>SDI Panel mount coupler</t>
         </is>
       </c>
-      <c r="B56" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="inlineStr">
+      <c r="B59" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="50" t="inlineStr">
         <is>
           <t>HD-SDI Cable, 1m - 4m</t>
         </is>
       </c>
-      <c r="B57" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="33" t="inlineStr">
+      <c r="B60" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="48" t="inlineStr">
         <is>
           <t>Slider - BMD Converter</t>
         </is>
       </c>
-      <c r="B58" s="34" t="n"/>
-      <c r="C58" s="35" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="15" t="inlineStr">
+      <c r="B61" s="49" t="n"/>
+      <c r="C61" s="49" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="50" t="inlineStr">
         <is>
           <t>SDI Panel mount coupler</t>
         </is>
       </c>
-      <c r="B59" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C59" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="15" t="inlineStr">
+      <c r="B62" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="50" t="inlineStr">
         <is>
           <t>HD-SDI Cable, 2m - 4m</t>
         </is>
       </c>
-      <c r="B60" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C60" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="33" t="inlineStr">
+      <c r="B63" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="48" t="inlineStr">
         <is>
           <t>Hub</t>
         </is>
       </c>
-      <c r="B61" s="34" t="n"/>
-      <c r="C61" s="35" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="15" t="inlineStr">
+      <c r="B64" s="49" t="n"/>
+      <c r="C64" s="49" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="50" t="inlineStr">
         <is>
           <t>Seeed Studio XIAO ESP32S3</t>
         </is>
       </c>
-      <c r="B62" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="33" t="inlineStr">
+      <c r="B65" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="48" t="inlineStr">
         <is>
           <t>Hub Display</t>
         </is>
       </c>
-      <c r="B63" s="34" t="n"/>
-      <c r="C63" s="35" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="15" t="inlineStr">
+      <c r="B66" s="49" t="n"/>
+      <c r="C66" s="49" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="50" t="inlineStr">
         <is>
           <t>Waveshare ESP32-S3 7inch Capacitive Touch LCD</t>
         </is>
       </c>
-      <c r="B64" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="15" t="inlineStr">
+      <c r="B67" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="50" t="inlineStr">
         <is>
           <t>2.4GHz Antenna</t>
         </is>
       </c>
-      <c r="B65" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="15" t="inlineStr">
+      <c r="B68" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="50" t="inlineStr">
         <is>
           <t>U.FL Mini PCI to SMA Female 20cm Lead</t>
         </is>
       </c>
-      <c r="B66" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="15" t="inlineStr">
+      <c r="B69" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="50" t="inlineStr">
         <is>
           <t>USB-C Screw Hole Panel Mount</t>
         </is>
       </c>
-      <c r="B67" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="33" t="inlineStr">
+      <c r="B70" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="48" t="inlineStr">
         <is>
           <t>Misc</t>
         </is>
       </c>
-      <c r="B68" s="34" t="n"/>
-      <c r="C68" s="35" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="15" t="inlineStr">
+      <c r="B71" s="49" t="n"/>
+      <c r="C71" s="49" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="50" t="inlineStr">
         <is>
           <t>2 Core Wire - 30m, 20awg</t>
         </is>
       </c>
-      <c r="B69" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C69" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="15" t="inlineStr">
+      <c r="B72" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="50" t="inlineStr">
         <is>
           <t>4 Core Wire - 10m, 24awg</t>
         </is>
       </c>
-      <c r="B70" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C70" s="17" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="33" t="inlineStr">
+      <c r="B73" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" s="52" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="48" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="B71" s="34" t="n"/>
-      <c r="C71" s="35" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="15" t="inlineStr">
+      <c r="B74" s="49" t="n"/>
+      <c r="C74" s="49" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="50" t="inlineStr">
         <is>
           <t>UGREEN Video Capture Card HDMI to USB C 1080P 60FPS Capture (CV Tracking)</t>
         </is>
       </c>
-      <c r="B72" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C72" s="17" t="inlineStr">
+      <c r="B75" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" s="52" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
@@ -1823,19 +1937,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A63:C63"/>
     <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A61:C61"/>
     <mergeCell ref="A58:C58"/>
-    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A74:C74"/>
     <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A38:C38"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A64:C64"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
@@ -1865,15 +1979,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId39"/>
@@ -1882,20 +1996,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1907,7 +2023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN57"/>
+  <dimension ref="B2:AN57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="10.83203125" customWidth="1" style="41" min="1" max="1"/>
@@ -1949,7 +2065,6 @@
     <col width="10.83203125" customWidth="1" style="41" min="40" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="18" t="inlineStr">
         <is>
@@ -2470,10 +2585,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20">
       <c r="B20" s="18" t="inlineStr">
         <is>
@@ -3041,7 +3152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="B2:V35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="3.33203125" customWidth="1" min="1" max="1"/>
@@ -3050,7 +3161,6 @@
     <col width="8" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="57" customHeight="1">
       <c r="B2" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: correct the 1/4 UNC insert supplier link
Points at the insert that actually worked out best in use (B0B1F7NMJ5),
replacing the first link recorded for it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/assets/BoM.xlsx
+++ b/docs/assets/BoM.xlsx
@@ -180,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -378,11 +378,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -475,6 +519,8 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -903,8 +949,8 @@
           <t>Circuit</t>
         </is>
       </c>
-      <c r="B2" s="49" t="n"/>
-      <c r="C2" s="49" t="n"/>
+      <c r="B2" s="54" t="n"/>
+      <c r="C2" s="55" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="50" t="inlineStr">
@@ -1111,8 +1157,8 @@
           <t>Mount</t>
         </is>
       </c>
-      <c r="B16" s="49" t="n"/>
-      <c r="C16" s="49" t="n"/>
+      <c r="B16" s="54" t="n"/>
+      <c r="C16" s="55" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="50" t="inlineStr">
@@ -1345,8 +1391,8 @@
           <t>Mount - HDMI</t>
         </is>
       </c>
-      <c r="B32" s="49" t="n"/>
-      <c r="C32" s="49" t="n"/>
+      <c r="B32" s="54" t="n"/>
+      <c r="C32" s="55" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="50" t="inlineStr">
@@ -1384,8 +1430,8 @@
           <t>Mount - SDI</t>
         </is>
       </c>
-      <c r="B35" s="49" t="n"/>
-      <c r="C35" s="49" t="n"/>
+      <c r="B35" s="54" t="n"/>
+      <c r="C35" s="55" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="50" t="inlineStr">
@@ -1423,8 +1469,8 @@
           <t>Mount - BMD Converter</t>
         </is>
       </c>
-      <c r="B38" s="49" t="n"/>
-      <c r="C38" s="49" t="n"/>
+      <c r="B38" s="54" t="n"/>
+      <c r="C38" s="55" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="50" t="inlineStr">
@@ -1492,8 +1538,8 @@
           <t>Slider</t>
         </is>
       </c>
-      <c r="B43" s="49" t="n"/>
-      <c r="C43" s="49" t="n"/>
+      <c r="B43" s="54" t="n"/>
+      <c r="C43" s="55" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="50" t="inlineStr">
@@ -1668,8 +1714,8 @@
           <t>Slider - HDMI</t>
         </is>
       </c>
-      <c r="B55" s="49" t="n"/>
-      <c r="C55" s="49" t="n"/>
+      <c r="B55" s="54" t="n"/>
+      <c r="C55" s="55" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="50" t="inlineStr">
@@ -1707,8 +1753,8 @@
           <t>Slider - SDI</t>
         </is>
       </c>
-      <c r="B58" s="49" t="n"/>
-      <c r="C58" s="49" t="n"/>
+      <c r="B58" s="54" t="n"/>
+      <c r="C58" s="55" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="50" t="inlineStr">
@@ -1746,8 +1792,8 @@
           <t>Slider - BMD Converter</t>
         </is>
       </c>
-      <c r="B61" s="49" t="n"/>
-      <c r="C61" s="49" t="n"/>
+      <c r="B61" s="54" t="n"/>
+      <c r="C61" s="55" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="50" t="inlineStr">
@@ -1785,8 +1831,8 @@
           <t>Hub</t>
         </is>
       </c>
-      <c r="B64" s="49" t="n"/>
-      <c r="C64" s="49" t="n"/>
+      <c r="B64" s="54" t="n"/>
+      <c r="C64" s="55" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="50" t="inlineStr">
@@ -1809,8 +1855,8 @@
           <t>Hub Display</t>
         </is>
       </c>
-      <c r="B66" s="49" t="n"/>
-      <c r="C66" s="49" t="n"/>
+      <c r="B66" s="54" t="n"/>
+      <c r="C66" s="55" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="50" t="inlineStr">
@@ -1878,8 +1924,8 @@
           <t>Misc</t>
         </is>
       </c>
-      <c r="B71" s="49" t="n"/>
-      <c r="C71" s="49" t="n"/>
+      <c r="B71" s="54" t="n"/>
+      <c r="C71" s="55" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="50" t="inlineStr">
@@ -1917,8 +1963,8 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="B74" s="49" t="n"/>
-      <c r="C74" s="49" t="n"/>
+      <c r="B74" s="54" t="n"/>
+      <c r="C74" s="55" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="50" t="inlineStr">

</xml_diff>